<commit_message>
Unifying data in Excels
</commit_message>
<xml_diff>
--- a/2026-ECMFA/RQ1/results/experiment_run_gemini-2_5-flash.xlsx
+++ b/2026-ECMFA/RQ1/results/experiment_run_gemini-2_5-flash.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\proyectos\emf-kaizen-experiments\2026-ECMFA\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\emf-kaizen-experiments\2026-ECMFA\RQ1\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62D137BB-7754-4CFE-83C4-64E8617695E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D70544E9-4389-40A2-AE47-642990718297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="eval run syntax" sheetId="3" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="75">
   <si>
     <t>Meta-models</t>
   </si>
@@ -173,15 +173,6 @@
     <t>Missing reference</t>
   </si>
   <si>
-    <t>No response</t>
-  </si>
-  <si>
-    <t>Response shown as text in chat</t>
-  </si>
-  <si>
-    <t>Other errors</t>
-  </si>
-  <si>
     <t>Has some elements repeated from the current model, unnecesarily</t>
   </si>
   <si>
@@ -273,6 +264,9 @@
   </si>
   <si>
     <t>mediana</t>
+  </si>
+  <si>
+    <t>Incorrect intent</t>
   </si>
 </sst>
 </file>
@@ -1145,7 +1139,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.36328125" customWidth="1"/>
@@ -1154,18 +1148,18 @@
     <col min="4" max="11" width="12.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D3" s="29" t="s">
         <v>8</v>
       </c>
@@ -1183,7 +1177,7 @@
       </c>
       <c r="K3" s="32"/>
     </row>
-    <row r="4" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -1229,17 +1223,11 @@
       <c r="P4">
         <v>4</v>
       </c>
-      <c r="Q4">
-        <v>5</v>
-      </c>
-      <c r="R4">
-        <v>6</v>
-      </c>
-      <c r="S4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="Q4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="26" t="s">
         <v>1</v>
       </c>
@@ -1274,14 +1262,14 @@
         <v>1</v>
       </c>
       <c r="L5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="M5">
         <f>COUNTIF($D5:$K7,M4)</f>
         <v>14</v>
       </c>
       <c r="N5">
-        <f t="shared" ref="N5:R5" si="0">COUNTIF($D5:$K7,N4)</f>
+        <f t="shared" ref="N5:P5" si="0">COUNTIF($D5:$K7,N4)</f>
         <v>0</v>
       </c>
       <c r="O5">
@@ -1293,19 +1281,11 @@
         <v>0</v>
       </c>
       <c r="Q5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="S5">
-        <f>SUM(M5:R5)</f>
+        <f>SUM(M5:P5)</f>
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="27"/>
       <c r="B6" s="6" t="s">
         <v>3</v>
@@ -1338,14 +1318,14 @@
         <v>3</v>
       </c>
       <c r="L6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="M6">
         <f>100*M5/24</f>
         <v>58.333333333333336</v>
       </c>
       <c r="N6">
-        <f t="shared" ref="N6:R6" si="1">100*N5/24</f>
+        <f t="shared" ref="N6:P6" si="1">100*N5/24</f>
         <v>0</v>
       </c>
       <c r="O6">
@@ -1356,16 +1336,8 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="7" spans="1:17" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="28"/>
       <c r="B7" s="7" t="s">
         <v>4</v>
@@ -1398,7 +1370,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="33" t="s">
         <v>20</v>
       </c>
@@ -1433,14 +1405,14 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="M8">
         <f>COUNTIF($D8:$K10,M4)</f>
         <v>24</v>
       </c>
       <c r="N8">
-        <f t="shared" ref="N8:R8" si="2">COUNTIF($D8:$K10,N4)</f>
+        <f t="shared" ref="N8:P8" si="2">COUNTIF($D8:$K10,N4)</f>
         <v>0</v>
       </c>
       <c r="O8">
@@ -1452,19 +1424,11 @@
         <v>0</v>
       </c>
       <c r="Q8">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R8">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="S8">
-        <f>SUM(M8:R8)</f>
+        <f>SUM(M8:P8)</f>
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="34"/>
       <c r="B9" s="6" t="s">
         <v>3</v>
@@ -1497,14 +1461,14 @@
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="M9">
         <f>100*M8/24</f>
         <v>100</v>
       </c>
       <c r="N9">
-        <f t="shared" ref="N9:R9" si="3">100*N8/24</f>
+        <f t="shared" ref="N9:P9" si="3">100*N8/24</f>
         <v>0</v>
       </c>
       <c r="O9">
@@ -1515,16 +1479,8 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="Q9">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="R9">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="10" spans="1:17" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="35"/>
       <c r="B10" s="7" t="s">
         <v>4</v>
@@ -1557,7 +1513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="26" t="s">
         <v>2</v>
       </c>
@@ -1592,14 +1548,14 @@
         <v>1</v>
       </c>
       <c r="L11" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="M11">
         <f>COUNTIF($D11:$K13,M4)</f>
         <v>22</v>
       </c>
       <c r="N11">
-        <f t="shared" ref="N11:R11" si="4">COUNTIF($D11:$K13,N4)</f>
+        <f t="shared" ref="N11:P11" si="4">COUNTIF($D11:$K13,N4)</f>
         <v>1</v>
       </c>
       <c r="O11">
@@ -1611,19 +1567,11 @@
         <v>0</v>
       </c>
       <c r="Q11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="R11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="S11">
-        <f>SUM(M11:R11)</f>
+        <f>SUM(M11:P11)</f>
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="27"/>
       <c r="B12" s="6" t="s">
         <v>3</v>
@@ -1656,14 +1604,14 @@
         <v>1</v>
       </c>
       <c r="L12" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="M12">
         <f>100*M11/24</f>
         <v>91.666666666666671</v>
       </c>
       <c r="N12">
-        <f t="shared" ref="N12:R12" si="5">100*N11/24</f>
+        <f t="shared" ref="N12:P12" si="5">100*N11/24</f>
         <v>4.166666666666667</v>
       </c>
       <c r="O12">
@@ -1674,16 +1622,8 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q12">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R12">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="13" spans="1:17" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="28"/>
       <c r="B13" s="7" t="s">
         <v>4</v>
@@ -1716,7 +1656,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="26" t="s">
         <v>17</v>
       </c>
@@ -1751,14 +1691,14 @@
         <v>1</v>
       </c>
       <c r="L14" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="M14">
         <f>COUNTIF($D14:$K16,M4)</f>
         <v>22</v>
       </c>
       <c r="N14">
-        <f t="shared" ref="N14:R14" si="6">COUNTIF($D14:$K16,N4)</f>
+        <f t="shared" ref="N14:P14" si="6">COUNTIF($D14:$K16,N4)</f>
         <v>0</v>
       </c>
       <c r="O14">
@@ -1770,19 +1710,11 @@
         <v>0</v>
       </c>
       <c r="Q14">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R14">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="S14">
-        <f>SUM(M14:R14)</f>
+        <f>SUM(M14:P14)</f>
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="27"/>
       <c r="B15" s="6" t="s">
         <v>3</v>
@@ -1815,14 +1747,14 @@
         <v>1</v>
       </c>
       <c r="L15" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="M15">
         <f>100*M14/24</f>
         <v>91.666666666666671</v>
       </c>
       <c r="N15">
-        <f t="shared" ref="N15:R15" si="7">100*N14/24</f>
+        <f t="shared" ref="N15:P15" si="7">100*N14/24</f>
         <v>0</v>
       </c>
       <c r="O15">
@@ -1833,16 +1765,8 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="Q15">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="R15">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="16" spans="1:17" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="28"/>
       <c r="B16" s="7" t="s">
         <v>4</v>
@@ -1875,7 +1799,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="26" t="s">
         <v>19</v>
       </c>
@@ -1910,14 +1834,14 @@
         <v>3</v>
       </c>
       <c r="L17" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="M17">
         <f>COUNTIF($D17:$K19,M4)</f>
         <v>17</v>
       </c>
       <c r="N17">
-        <f t="shared" ref="N17:R17" si="8">COUNTIF($D17:$K19,N4)</f>
+        <f t="shared" ref="N17:P17" si="8">COUNTIF($D17:$K19,N4)</f>
         <v>0</v>
       </c>
       <c r="O17">
@@ -1929,19 +1853,11 @@
         <v>0</v>
       </c>
       <c r="Q17">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="R17">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="S17">
-        <f>SUM(M17:R17)</f>
+        <f>SUM(M17:P17)</f>
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="27"/>
       <c r="B18" s="6" t="s">
         <v>3</v>
@@ -1974,14 +1890,14 @@
         <v>3</v>
       </c>
       <c r="L18" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="M18">
         <f>100*M17/24</f>
         <v>70.833333333333329</v>
       </c>
       <c r="N18">
-        <f t="shared" ref="N18:R18" si="9">100*N17/24</f>
+        <f t="shared" ref="N18:P18" si="9">100*N17/24</f>
         <v>0</v>
       </c>
       <c r="O18">
@@ -1992,16 +1908,8 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="Q18">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="R18">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="19" spans="1:17" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="28"/>
       <c r="B19" s="7" t="s">
         <v>4</v>
@@ -2034,15 +1942,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
       <c r="E21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F21" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>39</v>
       </c>
@@ -2061,7 +1969,7 @@
         <v>82.5</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B23">
         <v>2</v>
       </c>
@@ -2069,15 +1977,15 @@
         <v>41</v>
       </c>
       <c r="E23">
-        <f t="shared" ref="E23:E27" si="10">COUNTIF(D$5:K$19,B23)</f>
+        <f t="shared" ref="E23:E25" si="10">COUNTIF(D$5:K$19,B23)</f>
         <v>1</v>
       </c>
       <c r="F23">
-        <f t="shared" ref="F23:F27" si="11">100*E23/(15*8)</f>
+        <f t="shared" ref="F23:F25" si="11">100*E23/(15*8)</f>
         <v>0.83333333333333337</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B24">
         <v>3</v>
       </c>
@@ -2093,50 +2001,18 @@
         <v>16.666666666666668</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B25">
         <v>4</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>43</v>
+        <v>74</v>
       </c>
       <c r="E25">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F25">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B26">
-        <v>5</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E26">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="F26">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B27">
-        <v>6</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E27">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="F27">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -2173,7 +2049,7 @@
         <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -2230,10 +2106,10 @@
         <v>16</v>
       </c>
       <c r="N4" s="23" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="O4" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2321,7 +2197,7 @@
         <v>2</v>
       </c>
       <c r="M6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="N6">
         <f t="shared" ref="N6:N7" si="0">COUNTIF(D$5:K$7,L6)</f>
@@ -2368,7 +2244,7 @@
         <v>3</v>
       </c>
       <c r="M7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="N7">
         <f t="shared" si="0"/>
@@ -2464,7 +2340,7 @@
         <v>2</v>
       </c>
       <c r="M9" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="N9">
         <f t="shared" ref="N9:N10" si="2">COUNTIF(D$8:K$10,L9)</f>
@@ -2511,7 +2387,7 @@
         <v>3</v>
       </c>
       <c r="M10" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="N10">
         <f t="shared" si="2"/>
@@ -2607,7 +2483,7 @@
         <v>2</v>
       </c>
       <c r="M12" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="N12">
         <f t="shared" ref="N12:N13" si="3">COUNTIF(D$11:K$13,L12)</f>
@@ -2654,7 +2530,7 @@
         <v>3</v>
       </c>
       <c r="M13" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="N13">
         <f t="shared" si="3"/>
@@ -2750,7 +2626,7 @@
         <v>2</v>
       </c>
       <c r="M15" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="N15">
         <f t="shared" ref="N15:N16" si="4">COUNTIF(D$14:K$16,L15)</f>
@@ -2797,7 +2673,7 @@
         <v>3</v>
       </c>
       <c r="M16" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="N16">
         <f t="shared" si="4"/>
@@ -2893,7 +2769,7 @@
         <v>2</v>
       </c>
       <c r="M18" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="N18">
         <f t="shared" ref="N18:N19" si="5">COUNTIF(D$17:K$19,L18)</f>
@@ -2940,7 +2816,7 @@
         <v>3</v>
       </c>
       <c r="M19" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="N19">
         <f t="shared" si="5"/>
@@ -2953,10 +2829,10 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="F21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G21" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.35">
@@ -2983,7 +2859,7 @@
         <v>2</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F23">
         <f>COUNTIF(D$5:K$19,B23)</f>
@@ -2999,7 +2875,7 @@
         <v>3</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F24">
         <f>COUNTIF(D$5:K$19,B24)</f>
@@ -3042,7 +2918,7 @@
         <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -3099,10 +2975,10 @@
         <v>16</v>
       </c>
       <c r="N4" s="23" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="O4" s="23" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3143,7 +3019,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="N5">
         <f>COUNTIF(D$5:K$7,L5)</f>
@@ -3190,7 +3066,7 @@
         <v>2</v>
       </c>
       <c r="M6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="N6">
         <f t="shared" ref="N6:N7" si="0">COUNTIF(D$5:K$7,L6)</f>
@@ -3237,7 +3113,7 @@
         <v>3</v>
       </c>
       <c r="M7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="N7">
         <f t="shared" si="0"/>
@@ -3286,7 +3162,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="N8">
         <f>COUNTIF(D$8:K$10,L8)</f>
@@ -3333,7 +3209,7 @@
         <v>2</v>
       </c>
       <c r="M9" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="N9">
         <f t="shared" ref="N9:N10" si="2">COUNTIF(D$8:K$10,L9)</f>
@@ -3380,7 +3256,7 @@
         <v>3</v>
       </c>
       <c r="M10" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="N10">
         <f t="shared" si="2"/>
@@ -3429,7 +3305,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="N11">
         <f>COUNTIF(D$11:K$13,L11)</f>
@@ -3476,7 +3352,7 @@
         <v>2</v>
       </c>
       <c r="M12" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="N12">
         <f t="shared" ref="N12:N13" si="3">COUNTIF(D$11:K$13,L12)</f>
@@ -3523,7 +3399,7 @@
         <v>3</v>
       </c>
       <c r="M13" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="N13">
         <f t="shared" si="3"/>
@@ -3572,7 +3448,7 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="N14">
         <f>COUNTIF(D$14:K$16,L14)</f>
@@ -3619,7 +3495,7 @@
         <v>2</v>
       </c>
       <c r="M15" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="N15">
         <f t="shared" ref="N15:N16" si="4">COUNTIF(D$14:K$16,L15)</f>
@@ -3666,7 +3542,7 @@
         <v>3</v>
       </c>
       <c r="M16" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="N16">
         <f t="shared" si="4"/>
@@ -3715,7 +3591,7 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="N17">
         <f>COUNTIF(D$17:K$19,L17)</f>
@@ -3762,7 +3638,7 @@
         <v>2</v>
       </c>
       <c r="M18" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="N18">
         <f t="shared" ref="N18:N19" si="5">COUNTIF(D$17:K$19,L18)</f>
@@ -3809,7 +3685,7 @@
         <v>3</v>
       </c>
       <c r="M19" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="N19">
         <f t="shared" si="5"/>
@@ -3822,10 +3698,10 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="D21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E21" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.35">
@@ -3836,7 +3712,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D22">
         <f>COUNTIF(D$5:K$19,B22)</f>
@@ -3852,7 +3728,7 @@
         <v>2</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D23">
         <f t="shared" ref="D23:D24" si="6">COUNTIF(D$5:K$19,B23)</f>
@@ -3868,7 +3744,7 @@
         <v>3</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D24">
         <f t="shared" si="6"/>
@@ -3911,7 +3787,7 @@
         <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -3933,7 +3809,7 @@
       </c>
       <c r="K3" s="32"/>
       <c r="M3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -3974,13 +3850,13 @@
         <v>8</v>
       </c>
       <c r="N4" s="21" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O4" s="21" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="P4" s="21" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4176,7 +4052,7 @@
         <v>3</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="M8">
         <f>SUM(M5:M7)</f>
@@ -4577,10 +4453,10 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="D21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E21" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
@@ -4591,7 +4467,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D22">
         <f>COUNTIF(D$5:K$19,B22)</f>
@@ -4607,7 +4483,7 @@
         <v>2</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D23">
         <f t="shared" ref="D23:D24" si="4">COUNTIF(D$5:K$19,B23)</f>
@@ -4623,7 +4499,7 @@
         <v>3</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D24">
         <f t="shared" si="4"/>
@@ -4666,7 +4542,7 @@
         <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -4688,7 +4564,7 @@
       </c>
       <c r="K3" s="32"/>
       <c r="M3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -4726,16 +4602,16 @@
         <v>16</v>
       </c>
       <c r="M4" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="N4" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="O4" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="P4" s="24" t="s">
         <v>67</v>
-      </c>
-      <c r="N4" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="O4" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="P4" s="24" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -5343,7 +5219,7 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B21">
         <f>SUM(D5:K19)/120</f>
@@ -5352,7 +5228,7 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B22">
         <f>MIN(D5:K19)</f>
@@ -5361,7 +5237,7 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B23">
         <f>MAX(D5:K19)</f>
@@ -5370,7 +5246,6 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A14:A16"/>
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="F3:G3"/>
@@ -5379,6 +5254,7 @@
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A14:A16"/>
   </mergeCells>
   <conditionalFormatting sqref="D5:K19">
     <cfRule type="colorScale" priority="1">
@@ -5412,7 +5288,7 @@
         <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -5434,7 +5310,7 @@
       </c>
       <c r="K3" s="32"/>
       <c r="M3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -5472,16 +5348,16 @@
         <v>16</v>
       </c>
       <c r="M4" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="N4" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="O4" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="P4" s="24" t="s">
         <v>67</v>
-      </c>
-      <c r="N4" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="O4" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="P4" s="24" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6089,7 +5965,7 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B21">
         <f>SUM(D5:K19)/120</f>
@@ -6098,7 +5974,7 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B22">
         <f>MIN(D5:K19)</f>
@@ -6107,7 +5983,7 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B23">
         <f>MAX(D5:K19)</f>
@@ -6158,7 +6034,7 @@
         <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -6180,7 +6056,7 @@
       </c>
       <c r="K3" s="39"/>
       <c r="M3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -6218,16 +6094,16 @@
         <v>16</v>
       </c>
       <c r="M4" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="N4" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="O4" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="P4" s="24" t="s">
         <v>67</v>
-      </c>
-      <c r="N4" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="O4" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="P4" s="24" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6835,7 +6711,7 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="L21" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="M21">
         <f>MEDIAN(D5:E19)</f>
@@ -6859,10 +6735,10 @@
         <v>39</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E22" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F22" s="25">
         <f>MEDIAN(D5:K19)</f>
@@ -6871,7 +6747,7 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E23" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F23" s="25">
         <f>MIN(D5:K19)</f>
@@ -6880,7 +6756,7 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="E24" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F24" s="25">
         <f>MAX(D5:K19)</f>

</xml_diff>